<commit_message>
fix(gui): fix status label updates and excel column parsing
The DigitalIndicator and ChannelIndicator classes were incorrectly updating
status_label instead of value_label when displaying status messages. This caused
status text to appear in the wrong UI element.

Additionally, improved Excel export conditional formatting to use regex when
parsing channel numbers from column names. This properly handles custom column
names like "CH1 (3.3VD)" by extracting only the numeric channel identifier.

Configuration for channel 1 (3.3VD) was also updated with correct AUTO range
and proper voltage thresholds (3.2-3.4V).
</commit_message>
<xml_diff>
--- a/B1ControlExtensionBoardv232_2026-01-29.xlsx
+++ b/B1ControlExtensionBoardv232_2026-01-29.xlsx
@@ -26,12 +26,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCFFCC"/>
+        <bgColor rgb="00CCFFCC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -52,9 +58,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -508,38 +515,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FAILED CH1 (3.3VD): -0.0010735 (expected: 150.0 - 180.0); CH2 (5.0VD): -0.0011545 (expected: 2.0 - 2.1); CH3 (12V): -0.0011599 (expected: 2.0 - 2.1); CH4 (7V): -0.0011203 (expected: 2.0 - 2.1); CH6: -0.0012311 (expected: 2.1 - 2.2); CH7: -0.0010862 (expected: 1.0 - 1.1)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>-0.0010735</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>-0.0011545</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>-0.0011599</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>-0.0011203</t>
+          <t>FAILED CH2 (5.0VD): -0.0001831 (expected: 2.0 - 2.1); CH3 (12V): -0.0004034 (expected: 2.0 - 2.1); CH4 (7V): -0.0002586 (expected: 2.0 - 2.1); CH6: -0.0003287 (expected: 2.1 - 2.2); CH7: -0.0003147 (expected: 1.0 - 1.1)</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>3.3012368</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>-0.0001831</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>-0.0004034</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>-0.0002586</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>-0.0012311</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>-0.0010862</t>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>-0.0003287</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>-0.0003147</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -549,7 +556,7 @@
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-01-29 17:19:06</t>
+          <t>2026-01-29 18:03:36</t>
         </is>
       </c>
     </row>
@@ -564,33 +571,33 @@
           <t>FAILED CH1 (3.3VD): -0.0010274 (expected: 150.0 - 180.0); CH2 (5.0VD): -0.0011233 (expected: 2.0 - 2.1); CH3 (12V): -0.0011114 (expected: 2.0 - 2.1); CH4 (7V): -0.0011605 (expected: 2.0 - 2.1); CH6: -0.0010832 (expected: 2.1 - 2.2); CH7: -0.0010537 (expected: 1.0 - 1.1)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>-0.0010274</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>-0.0011233</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>-0.0011114</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>-0.0011605</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>-0.0010832</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>-0.0010537</t>
         </is>

</xml_diff>

<commit_message>
feat(gui): add enhanced excel formatting
Apply enhanced formatting to exported Excel worksheets including:
- Bold headers with center alignment
- Cell borders for all data and header cells
- Auto-adjusted column widths based on content
</commit_message>
<xml_diff>
--- a/B1ControlExtensionBoardv232_2026-01-29.xlsx
+++ b/B1ControlExtensionBoardv232_2026-01-29.xlsx
@@ -17,13 +17,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -46,7 +51,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,14 +59,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,185 +452,202 @@
   </sheetPr>
   <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="272" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>QR</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>TEST RESULT</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>CH1 (3.3VD)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>CH2 (5.0VD)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CH3 (12V)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CH4 (7V)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>CH5</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>CH6</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>CH7</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>CH8</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>CH9</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>CH10</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>CH11</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>CH12</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Date/Time</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>PSN000006047</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>FAILED CH2 (5.0VD): -0.0001831 (expected: 2.0 - 2.1); CH3 (12V): -0.0004034 (expected: 2.0 - 2.1); CH4 (7V): -0.0002586 (expected: 2.0 - 2.1); CH6: -0.0003287 (expected: 2.1 - 2.2); CH7: -0.0003147 (expected: 1.0 - 1.1)</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>3.3012368</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>-0.0001831</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>-0.0004034</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>-0.0002586</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>-0.0003287</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>-0.0003147</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>2026-01-29 18:03:36</t>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>FAILED CH2 (5.0VD): -0.0006273 (expected: 2.0 - 2.1); CH3 (12V): -0.0006922 (expected: 2.0 - 2.1); CH4 (7V): -0.0004386 (expected: 2.0 - 2.1); CH6: -0.0002427 (expected: 2.1 - 2.2); CH7: -0.0002427 (expected: 1.0 - 1.1)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>3.3016205</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-0.0006273</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>-0.0006922</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>-0.0004386</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>-0.0002427</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>-0.0002427</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29 18:20:18</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>PSN000002178</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>FAILED CH1 (3.3VD): -0.0010274 (expected: 150.0 - 180.0); CH2 (5.0VD): -0.0011233 (expected: 2.0 - 2.1); CH3 (12V): -0.0011114 (expected: 2.0 - 2.1); CH4 (7V): -0.0011605 (expected: 2.0 - 2.1); CH6: -0.0010832 (expected: 2.1 - 2.2); CH7: -0.0010537 (expected: 1.0 - 1.1)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>-0.0010274</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>-0.0011233</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>-0.0011114</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>-0.0011605</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>-0.0010832</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>-0.0010537</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>2026-01-29 17:20:45</t>
         </is>

</xml_diff>

<commit_message>
docs(spec): add excel export requirements to spec
Add comprehensive requirements for Excel export functionality including:
- Excel export button placement and behavior
- Conditional formatting based on measurement thresholds
- Excel file format specifications and data handling
- Export error handling for various edge cases
- Color contrast requirements for readability
</commit_message>
<xml_diff>
--- a/B1ControlExtensionBoardv232_2026-01-29.xlsx
+++ b/B1ControlExtensionBoardv232_2026-01-29.xlsx
@@ -555,38 +555,38 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>FAILED CH2 (5.0VD): -0.0006273 (expected: 2.0 - 2.1); CH3 (12V): -0.0006922 (expected: 2.0 - 2.1); CH4 (7V): -0.0004386 (expected: 2.0 - 2.1); CH6: -0.0002427 (expected: 2.1 - 2.2); CH7: -0.0002427 (expected: 1.0 - 1.1)</t>
+          <t>FAILED CH2 (5.0VD): -0.0002437 (expected: 2.0 - 2.1); CH3 (12V): -0.0002765 (expected: 2.0 - 2.1); CH4 (7V): -0.0002750 (expected: 2.0 - 2.1); CH6: -0.0004657 (expected: 2.1 - 2.2); CH7: -0.0003592 (expected: 1.0 - 1.1)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>3.3016205</t>
+          <t>3.3019297</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-0.0006273</t>
+          <t>-0.0002437</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>-0.0006922</t>
+          <t>-0.0002765</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>-0.0004386</t>
+          <t>-0.0002750</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>-0.0002427</t>
+          <t>-0.0004657</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>-0.0002427</t>
+          <t>-0.0003592</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -596,7 +596,7 @@
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-29 18:20:18</t>
+          <t>2026-01-29 18:36:09</t>
         </is>
       </c>
     </row>

</xml_diff>